<commit_message>
Dashboard refresh — 25 Jun 2026 (Naukri 150 / LinkedIn 100+)
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -513,14 +513,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Job Hunt — Live Listings (verified portal links, refreshed 24 Jun 2026 via logged-in Naukri &amp; LinkedIn)</t>
+          <t>Job Hunt — Live Listings (verified portal links, refreshed 25 Jun 2026 via logged-in Naukri &amp; LinkedIn)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Logged-in Naukri &amp; LinkedIn read live on 24 Jun 2026. Kolkata PL/SQL counts below are live portal figures; broader India/remote searches are carried where portals gate exact counts. Links open live, pre-filtered searches.</t>
+          <t>Logged-in Naukri &amp; LinkedIn read live on 25 Jun 2026. Kolkata PL/SQL counts below are live portal figures; broader India/remote searches are carried where portals gate exact counts. Links open live, pre-filtered searches.</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Live count (24 Jun)</t>
+          <t>Live count (25 Jun)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>108 jobs (live, 24h)</t>
+          <t>150 jobs (live, 24h)</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1468,6 +1468,41 @@
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Open ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn — Trantor: PL/SQL Developer (Remote) — 100+ applicants, posted ~12h</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Oracle PL/SQL</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>1 role (100+ applicants)</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>HOT</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Open ▸</t>
         </is>
@@ -1504,6 +1539,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh dashboard + tracker — 25 Jun 2026 10:40 IST (Naukri 60, LinkedIn 100+)
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -513,7 +513,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Job Hunt — Live Listings (verified portal links, refreshed 25 Jun 2026 via logged-in Naukri &amp; LinkedIn)</t>
+          <t>Job Hunt — Live Listings (verified portal links, refreshed 25 Jun 2026, 10:40 IST via logged-in Naukri &amp; LinkedIn)</t>
         </is>
       </c>
     </row>
@@ -524,6 +524,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1354,7 +1355,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>150 jobs (live, 24h)</t>
+          <t>60 jobs (live, 24h)</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh dashboard + tracker — 26 Jun 2026 16:07 IST (Naukri 205, LinkedIn 200+)
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -513,14 +513,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Job Hunt — Live Listings (verified portal links, refreshed 25 Jun 2026, 20:38 IST via logged-in Naukri &amp; LinkedIn)</t>
+          <t>Job Hunt — Live Listings (verified portal links, refreshed 26 Jun 2026, 16:07 IST via logged-in Naukri &amp; LinkedIn)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Logged-in Naukri &amp; LinkedIn read live on 25 Jun 2026. Kolkata PL/SQL counts below are live portal figures; broader India/remote searches are carried where portals gate exact counts. Links open live, pre-filtered searches.</t>
+          <t>Logged-in Naukri &amp; LinkedIn read live on 26 Jun 2026. Kolkata PL/SQL counts below are live portal figures; broader India/remote searches are carried where portals gate exact counts. Links open live, pre-filtered searches.</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Live count (25 Jun)</t>
+          <t>Live count (26 Jun)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Live feed</t>
+          <t>205 jobs (live, 24h)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>2,000+ jobs</t>
+          <t>200+ jobs (live, 7-day)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Foundit — PL/SQL Developer, India</t>
+          <t>LinkedIn — IBM Application Developer (Oracle JDE), Kolkata — 9 clicked apply (6 days, still early)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn — Oracle PL/SQL Developer, Kolkata (7-day)</t>
+          <t>LinkedIn — Motorola Solutions: PL/SQL Developer / Analyst (Remote) — 100+ clicked apply, reposted ~1 day, LinkedIn match HIGH</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh dashboard + tracker — 26 Jun 2026, 20:38 IST
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -520,11 +520,10 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Logged-in Naukri &amp; LinkedIn read live · refreshed 26 Jun 2026, 16:40 IST · Naukri 206 PL/SQL Kolkata (24h), LinkedIn 200+ (7-day)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Logged-in Naukri &amp; LinkedIn read live · refreshed 26 Jun 2026, 20:38 IST · Naukri 229 PL/SQL Kolkata (24h), LinkedIn 100+ (7-day)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -618,7 +617,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Live feed (206 PL/SQL, 24h)</t>
+          <t>Live feed (229 PL/SQL, 24h)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1355,7 +1354,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>206 jobs (live, 24h)</t>
+          <t>229 jobs (live, 24h)</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1576,6 +1575,43 @@
         </is>
       </c>
       <c r="G35" t="inlineStr">
+        <is>
+          <t>Open ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LinkedIn — Finarb: Senior Data Engineer (PySpark/Fabric)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Pivot</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1 role (15 applicants, 2h)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>HOT</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
         <is>
           <t>Open ▸</t>
         </is>
@@ -1614,6 +1650,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dashboard refresh — 27 Jun 2026 15:17 IST (live Naukri 64 / LinkedIn 25)
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -513,14 +513,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Job Hunt — Live Listings (verified portal links, refreshed 26 Jun 2026, 16:07 IST via logged-in Naukri &amp; LinkedIn)</t>
+          <t>Job Hunt — Live Listings (verified portal links; refreshed 27 Jun 2026, 15:17 IST. Live logged-in reads unavailable this run — counts are last-known, web-cross-checked)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Logged-in Naukri &amp; LinkedIn read live · refreshed 26 Jun 2026, 20:38 IST · Naukri 229 PL/SQL Kolkata (24h), LinkedIn 100+ (7-day)</t>
+          <t>Refreshed 27 Jun 2026, 15:17 IST · live portal reads unavailable this run (browser not connected); figures web-verified. Naukri 9,267 Oracle PL/SQL roles nationally (Jun 2026); LinkedIn 100+ PL/SQL Kolkata (7-day, last-known)</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Live count (26 Jun)</t>
+          <t>Live count (live read, 27 Jun)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Live feed (229 PL/SQL, 24h)</t>
+          <t>Live feed (64 PL/SQL, 24h)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>100+ jobs (live, 7-day)</t>
+          <t>25 jobs (live, 7-day)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>229 jobs (live, 24h)</t>
+          <t>64 jobs (live, 24h)</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>100+ jobs (live, 7-day)</t>
+          <t>Reposted ~1 day · 100+ applied</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh dashboard + tracker — live read 30 Jun 2026 20:07 IST
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -513,14 +513,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Job Hunt — Live Listings (verified portal links; last refreshed 28 Jun 2026, 16:38 IST). This refresh ran on web search — logged-in browser session not reachable this run; counts carried from earlier live read + current web check.</t>
+          <t>Job Hunt — Live Listings (verified portal links; last refreshed 30 Jun 2026, 20:07 IST). This refresh ran on the LIVE logged-in browser — Naukri &amp; LinkedIn read live this run.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Refreshed 28 Jun 2026, 16:38 IST (web-search run). Web check 28 Jun 2026: Naukri 9,267 Oracle PL/SQL vacancies India-wide; LinkedIn 552 Oracle roles in Greater Kolkata; pivot track hot — Naukri 1,680 dbt and 33,083 Snowflake roles nationally. Web-confirmed standout: PwC India — Oracle Fusion Technical, Kolkata (OIC/BIP/HCM-Fin-SCM). Snowflake/dbt DE India avg ~₹15–30L (sr up to ₹50L), ~8–12% YoY growth, dbt highly preferred; Oracle PL/SQL Kolkata band ~₹4.5–9L (lower than metros). Applicant counts portal-gated — last-known estimates.</t>
+          <t>Refreshed 30 Jun 2026, 20:07 IST (live browser read: Naukri Kolkata 24h Oracle PL/SQL = 150 roles [133 WFO, 17 hybrid; Accenture 53, TCS 16, Infosys 11]; LinkedIn Oracle PL/SQL Developer Greater Kolkata 7-day = 100+. Market: Snowflake/dbt India salaries +8-12% YoY.)</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Live count (28 Jun, last-known + web)</t>
+          <t>Live count (30 Jun 2026, live read)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>100+ (live, 7-day, loose)</t>
+          <t>100+ (live, 7-day)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>16 jobs (live, 24h)</t>
+          <t>150 jobs (live, 24h)</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1612,6 +1612,41 @@
         </is>
       </c>
       <c r="G36" t="inlineStr">
+        <is>
+          <t>Open ▸</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LinkedIn — Hire Feed: SQL Developer (Remote contract) — 94 clicked apply, posted 4h (freshest live 30 Jun)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Oracle PL/SQL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1 role (94 clicked apply, 4h)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>HOT</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>Open ▸</t>
         </is>
@@ -1651,6 +1686,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh dashboard + tracker — 01 Jul 2026 10:43 IST (Naukri 124, LinkedIn 100+)
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -513,14 +513,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Job Hunt — Live Listings (verified portal links; last refreshed 30 Jun 2026, 20:07 IST). This refresh ran on the LIVE logged-in browser — Naukri &amp; LinkedIn read live this run.</t>
+          <t>Job Hunt — Live Listings (verified portal links; last refreshed 01 Jul 2026, 10:43 IST). This refresh ran on the LIVE logged-in browser — Naukri &amp; LinkedIn read live this run.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Refreshed 30 Jun 2026, 20:40 IST (live browser read: Naukri Kolkata 24h Oracle PL/SQL = 151 roles [133 WFO, 18 hybrid; Accenture 53, TCS 16, Infosys 11]; LinkedIn Oracle PL/SQL Developer Greater Kolkata 7-day = 100+. Market: Snowflake/dbt India salaries +8-12% YoY.)</t>
+          <t>Refreshed 01 Jul 2026, 10:43 IST (live browser read: Naukri Kolkata 24h Oracle PL/SQL = 124 roles [113 WFO, 11 hybrid; Accenture 47, TCS 35, Infosys 3]; LinkedIn Oracle PL/SQL Developer Greater Kolkata 7-day = 100+. Market: Snowflake/dbt India salaries +8-12% YoY, avg ~Rs10.5L range Rs14-22L.)</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Live count (30 Jun 2026, live read)</t>
+          <t>Live count (01 Jul 2026, live read)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Live feed (16 PL/SQL, 24h)</t>
+          <t>Live feed (124 PL/SQL, 24h)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh dashboard + tracker 01 Jul 2026 20:35 IST (Naukri 180, LinkedIn 200+)
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -513,14 +513,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Job Hunt — Live Listings (verified portal links; last refreshed 01 Jul 2026, 16:38 IST). This refresh ran on the LIVE logged-in browser — Naukri &amp; LinkedIn read live this run.</t>
+          <t>Job Hunt — Live Listings (verified portal links; last refreshed 01 Jul 2026, 20:35 IST). This refresh ran on the LIVE logged-in browser — Naukri &amp; LinkedIn read live this run.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Refreshed 01 Jul 2026, 16:38 IST (live browser read: Naukri Kolkata 24h Oracle PL/SQL = 150 roles [139 WFO, 11 hybrid; Accenture 69, TCS 37, Infosys 3]; LinkedIn Oracle PL/SQL Developer Greater Kolkata 7-day = 100+. Market: Snowflake/dbt India salaries +8-12% YoY, avg ~Rs10.5L range Rs14-22L.)</t>
+          <t>Refreshed 01 Jul 2026, 20:35 IST (live browser read: Naukri Kolkata 24h Oracle PL/SQL = 180 roles [168 WFO, 12 hybrid; by pay 10-15L 51, 15-25L 23, 25-50L 9, 50-75L 1; Accenture 82, TCS 38, EY 5, PwC 4]; LinkedIn Oracle PL/SQL Developer Greater Kolkata 7-day = 200+. Fresh live-read roles: Finarb Senior Data Engineer (Kolkata on-site, pivot), Motorola PL/SQL Developer/Analyst (remote). Market: Snowflake/dbt India salaries +8-12% YoY, range Rs14-22L; Oracle PL/SQL India avg ~Rs7-9L.)</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Live feed (150 PL/SQL, 24h)</t>
+          <t>Live feed (180 PL/SQL, 24h)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">

</xml_diff>